<commit_message>
Regenerate results with the updated test titles
</commit_message>
<xml_diff>
--- a/workpapers/change-operations-workpaper.xlsx
+++ b/workpapers/change-operations-workpaper.xlsx
@@ -706,7 +706,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-28 02:11 UTC</t>
+          <t>2026-10-28 02:24 UTC</t>
         </is>
       </c>
     </row>
@@ -7453,12 +7453,12 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Only authorised people can sign in to the servers</t>
+          <t>Only authorised people can sign in to the servers and the PC</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Standard 5.1</t>
+          <t>Standard 5.1, 5.4</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -7506,12 +7506,12 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Administrator rights on the servers are limited to IT-Server-Admins</t>
+          <t>Administrator rights on the servers and the PC are limited as required</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Standard 5.2</t>
+          <t>Standard 5.2, 5.4</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -8301,7 +8301,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Server clocks are synchronised</t>
+          <t>Server and PC clocks are synchronised</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -8686,7 +8686,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OP-06: Server clocks are synchronised</t>
+          <t>OP-06: Server and PC clocks are synchronised</t>
         </is>
       </c>
     </row>
@@ -8738,7 +8738,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Control objective</t>
@@ -8746,7 +8746,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Every server keeps the correct time, so logs can be relied on and Kerberos sign in works.</t>
+          <t>Every server and PC keeps the correct time, so logs can be relied on and Kerberos sign in works.</t>
         </is>
       </c>
     </row>
@@ -8758,7 +8758,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Confirm each server synchronises with a time source and was within 5 seconds of it when the evidence was collected. Consider anything seen during fieldwork that shows the clock was wrong at other times.</t>
+          <t>Confirm each machine synchronises with a time source and was within 5 seconds of it when the evidence was collected. Consider anything seen during fieldwork that shows the clock was wrong at other times.</t>
         </is>
       </c>
     </row>
@@ -8770,7 +8770,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Both Linux servers</t>
+          <t>Both Linux servers and the PC</t>
         </is>
       </c>
     </row>
@@ -8982,7 +8982,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Known security weaknesses in the servers' software are fixed promptly.</t>
+          <t>Known security weaknesses in the software on the servers and the PC are fixed promptly.</t>
         </is>
       </c>
     </row>
@@ -9006,7 +9006,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Both Linux servers</t>
+          <t>Both Linux servers and the PC</t>
         </is>
       </c>
     </row>
@@ -11986,7 +11986,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AC-15: Only authorised people can sign in to the servers</t>
+          <t>AC-15: Only authorised people can sign in to the servers and the PC</t>
         </is>
       </c>
     </row>
@@ -11998,7 +11998,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Standard 5.1</t>
+          <t>Standard 5.1, 5.4</t>
         </is>
       </c>
     </row>
@@ -12062,7 +12062,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Population</t>
@@ -12070,7 +12070,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Every local account on both Linux servers, and the domain sign in setting on the app server</t>
+          <t>Every local account on both Linux servers and the PC, and the domain sign in setting on the app server</t>
         </is>
       </c>
     </row>
@@ -12266,7 +12266,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AC-16: Administrator rights on the servers are limited to IT-Server-Admins</t>
+          <t>AC-16: Administrator rights on the servers and the PC are limited as required</t>
         </is>
       </c>
     </row>
@@ -12278,7 +12278,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Standard 5.2</t>
+          <t>Standard 5.2, 5.4</t>
         </is>
       </c>
     </row>
@@ -12330,7 +12330,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
+    <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Test procedure</t>
@@ -12338,11 +12338,11 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>For every sudo rule on each server, record who it covers and what it allows. Full rights are allowed only through IT-Server-Admins. Rights limited to the deployment tool are allowed for Change-Deployers. A rule granted to a person directly, or one that does not ask for a password, is an exception unless the exception register covers it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1">
+          <t>For every sudo rule on each server, record who it covers and what it allows. Full rights are allowed only through IT-Server-Admins. Rights limited to the deployment tool are allowed for Change-Deployers. A rule granted to a person directly, or one that does not ask for a password, is an exception unless the exception register covers it. On the PC, any member of the local Administrators group other than Domain Admins and the disabled built in Administrator is an exception.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Population</t>
@@ -12350,7 +12350,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Every sudo rule on both Linux servers and every account it covers</t>
+          <t>Every sudo rule on both Linux servers and every account it covers, and every member of the PC's local Administrators group</t>
         </is>
       </c>
     </row>

</xml_diff>